<commit_message>
Fix README (complete instructions, fix broken links) and clean up requirements.txt
</commit_message>
<xml_diff>
--- a/crypto_history.xlsx
+++ b/crypto_history.xlsx
@@ -78,13 +78,13 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="000E622F"/>
+      <color rgb="009C0006"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="009C0006"/>
+      <color rgb="000E622F"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -541,10 +541,10 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="68" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -557,7 +557,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Automated pipeline telemetry — Generated on 2026-06-13 21:39:57</t>
+          <t>Automated pipeline telemetry — Generated on 2026-07-13 08:08:00</t>
         </is>
       </c>
     </row>
@@ -579,13 +579,13 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>25 Rows</t>
+          <t>115 Rows</t>
         </is>
       </c>
       <c r="B5" s="4" t="n"/>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>5 Unique Coins</t>
+          <t>6 Unique Coins</t>
         </is>
       </c>
       <c r="E5" s="4" t="n"/>
@@ -633,19 +633,19 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>NEAR Protocol</t>
+          <t>Solana</t>
         </is>
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>NEAR</t>
+          <t>SOL</t>
         </is>
       </c>
       <c r="D9" s="11" t="n">
-        <v>2.12</v>
+        <v>76.09</v>
       </c>
       <c r="E9" s="12" t="n">
-        <v>0.0424315</v>
+        <v>-0.0079445</v>
       </c>
     </row>
     <row r="10">
@@ -656,19 +656,19 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>Ethereum</t>
+          <t>Gram (prev. Toncoin)</t>
         </is>
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t>ETH</t>
+          <t>GRAM</t>
         </is>
       </c>
       <c r="D10" s="11" t="n">
-        <v>1680.3</v>
+        <v>1.6</v>
       </c>
       <c r="E10" s="12" t="n">
-        <v>0.0061836</v>
+        <v>-0.0334631</v>
       </c>
     </row>
   </sheetData>
@@ -688,10 +688,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
@@ -757,7 +757,7 @@
       <c r="E2" s="15" t="n">
         <v>28045462304</v>
       </c>
-      <c r="F2" s="16" t="n">
+      <c r="F2" s="12" t="n">
         <v>-0.000982</v>
       </c>
       <c r="G2" s="10" t="inlineStr">
@@ -769,116 +769,116 @@
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>Ethereum</t>
+          <t>Bitcoin</t>
         </is>
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>ETH</t>
+          <t>BTC</t>
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>1665.88</v>
+        <v>63613</v>
       </c>
       <c r="D3" s="15" t="n">
-        <v>201062160812</v>
+        <v>1274985882212</v>
       </c>
       <c r="E3" s="15" t="n">
-        <v>10810428629</v>
-      </c>
-      <c r="F3" s="16" t="n">
-        <v>-0.0106042</v>
+        <v>28045462304</v>
+      </c>
+      <c r="F3" s="12" t="n">
+        <v>-0.000982</v>
       </c>
       <c r="G3" s="10" t="inlineStr">
         <is>
-          <t>2026-06-12 22:36:14</t>
+          <t>2026-06-12 22:36:35</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>Solana</t>
+          <t>Bitcoin</t>
         </is>
       </c>
       <c r="B4" s="10" t="inlineStr">
         <is>
-          <t>SOL</t>
+          <t>BTC</t>
         </is>
       </c>
       <c r="C4" s="11" t="n">
-        <v>67.06999999999999</v>
+        <v>63682</v>
       </c>
       <c r="D4" s="15" t="n">
-        <v>38891640092</v>
+        <v>1276501384230</v>
       </c>
       <c r="E4" s="15" t="n">
-        <v>2789772399</v>
-      </c>
-      <c r="F4" s="12" t="n">
-        <v>0.0002204</v>
+        <v>27587409210</v>
+      </c>
+      <c r="F4" s="16" t="n">
+        <v>0.0001127</v>
       </c>
       <c r="G4" s="10" t="inlineStr">
         <is>
-          <t>2026-06-12 22:36:14</t>
+          <t>2026-06-12 22:43:27</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>Toncoin</t>
+          <t>Bitcoin</t>
         </is>
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>TON</t>
+          <t>BTC</t>
         </is>
       </c>
       <c r="C5" s="11" t="n">
-        <v>1.68</v>
+        <v>63682</v>
       </c>
       <c r="D5" s="15" t="n">
-        <v>4496794507</v>
+        <v>1276501384230</v>
       </c>
       <c r="E5" s="15" t="n">
-        <v>228774793</v>
+        <v>27587409210</v>
       </c>
       <c r="F5" s="16" t="n">
-        <v>-0.009129399999999999</v>
+        <v>0.0001127</v>
       </c>
       <c r="G5" s="10" t="inlineStr">
         <is>
-          <t>2026-06-12 22:36:14</t>
+          <t>2026-06-12 22:44:06</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>NEAR Protocol</t>
+          <t>Bitcoin</t>
         </is>
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>NEAR</t>
+          <t>BTC</t>
         </is>
       </c>
       <c r="C6" s="11" t="n">
-        <v>2.03</v>
+        <v>64212</v>
       </c>
       <c r="D6" s="15" t="n">
-        <v>2629686181</v>
+        <v>1286604959760</v>
       </c>
       <c r="E6" s="15" t="n">
-        <v>386759513</v>
+        <v>17930584160</v>
       </c>
       <c r="F6" s="16" t="n">
-        <v>-0.0156479</v>
+        <v>0.0069402</v>
       </c>
       <c r="G6" s="10" t="inlineStr">
         <is>
-          <t>2026-06-12 22:36:14</t>
+          <t>2026-06-13 21:39:57</t>
         </is>
       </c>
     </row>
@@ -894,136 +894,136 @@
         </is>
       </c>
       <c r="C7" s="11" t="n">
-        <v>63613</v>
+        <v>64158</v>
       </c>
       <c r="D7" s="15" t="n">
-        <v>1274985882212</v>
+        <v>1285564163013</v>
       </c>
       <c r="E7" s="15" t="n">
-        <v>28045462304</v>
+        <v>17694672759</v>
       </c>
       <c r="F7" s="16" t="n">
-        <v>-0.000982</v>
+        <v>0.0069492</v>
       </c>
       <c r="G7" s="10" t="inlineStr">
         <is>
-          <t>2026-06-12 22:36:35</t>
+          <t>2026-06-13 22:04:12</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>Ethereum</t>
+          <t>Bitcoin</t>
         </is>
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>ETH</t>
+          <t>BTC</t>
         </is>
       </c>
       <c r="C8" s="11" t="n">
-        <v>1665.88</v>
+        <v>65648</v>
       </c>
       <c r="D8" s="15" t="n">
-        <v>201062160812</v>
+        <v>1315764696145</v>
       </c>
       <c r="E8" s="15" t="n">
-        <v>10810428629</v>
+        <v>26120612925</v>
       </c>
       <c r="F8" s="16" t="n">
-        <v>-0.0106042</v>
+        <v>0.0189692</v>
       </c>
       <c r="G8" s="10" t="inlineStr">
         <is>
-          <t>2026-06-12 22:36:35</t>
+          <t>2026-06-15 11:58:38</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>Solana</t>
+          <t>Bitcoin</t>
         </is>
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>SOL</t>
+          <t>BTC</t>
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>67.06999999999999</v>
+        <v>62771</v>
       </c>
       <c r="D9" s="15" t="n">
-        <v>38891640092</v>
+        <v>1257926256203</v>
       </c>
       <c r="E9" s="15" t="n">
-        <v>2789772399</v>
+        <v>30165495087</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>0.0002204</v>
+        <v>-0.02589</v>
       </c>
       <c r="G9" s="10" t="inlineStr">
         <is>
-          <t>2026-06-12 22:36:35</t>
+          <t>2026-06-19 02:25:31</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>Toncoin</t>
+          <t>Bitcoin</t>
         </is>
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>TON</t>
+          <t>BTC</t>
         </is>
       </c>
       <c r="C10" s="11" t="n">
-        <v>1.68</v>
+        <v>62554</v>
       </c>
       <c r="D10" s="15" t="n">
-        <v>4496794507</v>
+        <v>1253892884190</v>
       </c>
       <c r="E10" s="15" t="n">
-        <v>228774793</v>
-      </c>
-      <c r="F10" s="16" t="n">
-        <v>-0.009129399999999999</v>
+        <v>29552578629</v>
+      </c>
+      <c r="F10" s="12" t="n">
+        <v>-0.0177444</v>
       </c>
       <c r="G10" s="10" t="inlineStr">
         <is>
-          <t>2026-06-12 22:36:35</t>
+          <t>2026-06-19 08:07:46</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>NEAR Protocol</t>
+          <t>Bitcoin</t>
         </is>
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>NEAR</t>
+          <t>BTC</t>
         </is>
       </c>
       <c r="C11" s="11" t="n">
-        <v>2.03</v>
+        <v>62985</v>
       </c>
       <c r="D11" s="15" t="n">
-        <v>2629686181</v>
+        <v>1263623120091</v>
       </c>
       <c r="E11" s="15" t="n">
-        <v>386759513</v>
+        <v>25183007618</v>
       </c>
       <c r="F11" s="16" t="n">
-        <v>-0.0156479</v>
+        <v>0.0048779</v>
       </c>
       <c r="G11" s="10" t="inlineStr">
         <is>
-          <t>2026-06-12 22:36:35</t>
+          <t>2026-06-19 21:42:06</t>
         </is>
       </c>
     </row>
@@ -1039,20 +1039,20 @@
         </is>
       </c>
       <c r="C12" s="11" t="n">
-        <v>63682</v>
+        <v>62985</v>
       </c>
       <c r="D12" s="15" t="n">
-        <v>1276501384230</v>
+        <v>1263623120091</v>
       </c>
       <c r="E12" s="15" t="n">
-        <v>27587409210</v>
-      </c>
-      <c r="F12" s="12" t="n">
-        <v>0.0001127</v>
+        <v>25183007618</v>
+      </c>
+      <c r="F12" s="16" t="n">
+        <v>0.0048779</v>
       </c>
       <c r="G12" s="10" t="inlineStr">
         <is>
-          <t>2026-06-12 22:43:27</t>
+          <t>2026-06-19 21:42:26</t>
         </is>
       </c>
     </row>
@@ -1068,74 +1068,74 @@
         </is>
       </c>
       <c r="C13" s="11" t="n">
-        <v>1667.49</v>
+        <v>1665.88</v>
       </c>
       <c r="D13" s="15" t="n">
-        <v>201282979948</v>
+        <v>201062160812</v>
       </c>
       <c r="E13" s="15" t="n">
-        <v>10360835032</v>
-      </c>
-      <c r="F13" s="16" t="n">
-        <v>-0.0106758</v>
+        <v>10810428629</v>
+      </c>
+      <c r="F13" s="12" t="n">
+        <v>-0.0106042</v>
       </c>
       <c r="G13" s="10" t="inlineStr">
         <is>
-          <t>2026-06-12 22:43:27</t>
+          <t>2026-06-12 22:36:14</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>Solana</t>
+          <t>Ethereum</t>
         </is>
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>SOL</t>
+          <t>ETH</t>
         </is>
       </c>
       <c r="C14" s="11" t="n">
-        <v>67.11</v>
+        <v>1665.88</v>
       </c>
       <c r="D14" s="15" t="n">
-        <v>38918087648</v>
+        <v>201062160812</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>2762112454</v>
+        <v>10810428629</v>
       </c>
       <c r="F14" s="12" t="n">
-        <v>0.000721</v>
+        <v>-0.0106042</v>
       </c>
       <c r="G14" s="10" t="inlineStr">
         <is>
-          <t>2026-06-12 22:43:27</t>
+          <t>2026-06-12 22:36:35</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>Toncoin</t>
+          <t>Ethereum</t>
         </is>
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>TON</t>
+          <t>ETH</t>
         </is>
       </c>
       <c r="C15" s="11" t="n">
-        <v>1.68</v>
+        <v>1667.49</v>
       </c>
       <c r="D15" s="15" t="n">
-        <v>4505181149</v>
+        <v>201282979948</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>229295333</v>
-      </c>
-      <c r="F15" s="16" t="n">
-        <v>-0.0063561</v>
+        <v>10360835032</v>
+      </c>
+      <c r="F15" s="12" t="n">
+        <v>-0.0106758</v>
       </c>
       <c r="G15" s="10" t="inlineStr">
         <is>
@@ -1146,58 +1146,58 @@
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>NEAR Protocol</t>
+          <t>Ethereum</t>
         </is>
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>NEAR</t>
+          <t>ETH</t>
         </is>
       </c>
       <c r="C16" s="11" t="n">
-        <v>2.03</v>
+        <v>1667.49</v>
       </c>
       <c r="D16" s="15" t="n">
-        <v>2638539801</v>
+        <v>201282979948</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>387461086</v>
-      </c>
-      <c r="F16" s="16" t="n">
-        <v>-0.0137975</v>
+        <v>10360835032</v>
+      </c>
+      <c r="F16" s="12" t="n">
+        <v>-0.0106758</v>
       </c>
       <c r="G16" s="10" t="inlineStr">
         <is>
-          <t>2026-06-12 22:43:27</t>
+          <t>2026-06-12 22:44:06</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>Bitcoin</t>
+          <t>Ethereum</t>
         </is>
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>BTC</t>
+          <t>ETH</t>
         </is>
       </c>
       <c r="C17" s="11" t="n">
-        <v>63682</v>
+        <v>1680.3</v>
       </c>
       <c r="D17" s="15" t="n">
-        <v>1276501384230</v>
+        <v>202700190893</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>27587409210</v>
-      </c>
-      <c r="F17" s="12" t="n">
-        <v>0.0001127</v>
+        <v>6329745882</v>
+      </c>
+      <c r="F17" s="16" t="n">
+        <v>0.0061836</v>
       </c>
       <c r="G17" s="10" t="inlineStr">
         <is>
-          <t>2026-06-12 22:44:06</t>
+          <t>2026-06-13 21:39:57</t>
         </is>
       </c>
     </row>
@@ -1213,136 +1213,136 @@
         </is>
       </c>
       <c r="C18" s="11" t="n">
-        <v>1667.49</v>
+        <v>1678.18</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>201282979948</v>
+        <v>202487435478</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>10360835032</v>
+        <v>6217595514</v>
       </c>
       <c r="F18" s="16" t="n">
-        <v>-0.0106758</v>
+        <v>0.0059298</v>
       </c>
       <c r="G18" s="10" t="inlineStr">
         <is>
-          <t>2026-06-12 22:44:06</t>
+          <t>2026-06-13 22:04:12</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>Solana</t>
+          <t>Ethereum</t>
         </is>
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>SOL</t>
+          <t>ETH</t>
         </is>
       </c>
       <c r="C19" s="11" t="n">
-        <v>67.11</v>
+        <v>1719.56</v>
       </c>
       <c r="D19" s="15" t="n">
-        <v>38918087648</v>
+        <v>207521752295</v>
       </c>
       <c r="E19" s="15" t="n">
-        <v>2762112454</v>
-      </c>
-      <c r="F19" s="12" t="n">
-        <v>0.000721</v>
+        <v>9493166557</v>
+      </c>
+      <c r="F19" s="16" t="n">
+        <v>0.026796</v>
       </c>
       <c r="G19" s="10" t="inlineStr">
         <is>
-          <t>2026-06-12 22:44:06</t>
+          <t>2026-06-15 11:58:38</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>Toncoin</t>
+          <t>Ethereum</t>
         </is>
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>TON</t>
+          <t>ETH</t>
         </is>
       </c>
       <c r="C20" s="11" t="n">
-        <v>1.68</v>
+        <v>1705.72</v>
       </c>
       <c r="D20" s="15" t="n">
-        <v>4505181149</v>
+        <v>205744973182</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>229295333</v>
-      </c>
-      <c r="F20" s="16" t="n">
-        <v>-0.0063561</v>
+        <v>12244401675</v>
+      </c>
+      <c r="F20" s="12" t="n">
+        <v>-0.0247926</v>
       </c>
       <c r="G20" s="10" t="inlineStr">
         <is>
-          <t>2026-06-12 22:44:06</t>
+          <t>2026-06-19 02:25:31</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>NEAR Protocol</t>
+          <t>Ethereum</t>
         </is>
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>NEAR</t>
+          <t>ETH</t>
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>2.03</v>
+        <v>1692.6</v>
       </c>
       <c r="D21" s="15" t="n">
-        <v>2638539801</v>
+        <v>204251518291</v>
       </c>
       <c r="E21" s="15" t="n">
-        <v>387461086</v>
-      </c>
-      <c r="F21" s="16" t="n">
-        <v>-0.0137975</v>
+        <v>11972438540</v>
+      </c>
+      <c r="F21" s="12" t="n">
+        <v>-0.017122</v>
       </c>
       <c r="G21" s="10" t="inlineStr">
         <is>
-          <t>2026-06-12 22:44:06</t>
+          <t>2026-06-19 08:07:46</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="14" t="inlineStr">
         <is>
-          <t>Bitcoin</t>
+          <t>Ethereum</t>
         </is>
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>BTC</t>
+          <t>ETH</t>
         </is>
       </c>
       <c r="C22" s="11" t="n">
-        <v>64212</v>
+        <v>1699.03</v>
       </c>
       <c r="D22" s="15" t="n">
-        <v>1286604959760</v>
+        <v>205204307648</v>
       </c>
       <c r="E22" s="15" t="n">
-        <v>17930584160</v>
-      </c>
-      <c r="F22" s="12" t="n">
-        <v>0.0069402</v>
+        <v>9085244988</v>
+      </c>
+      <c r="F22" s="16" t="n">
+        <v>0.0095683</v>
       </c>
       <c r="G22" s="10" t="inlineStr">
         <is>
-          <t>2026-06-13 21:39:57</t>
+          <t>2026-06-19 21:42:06</t>
         </is>
       </c>
     </row>
@@ -1358,107 +1358,2717 @@
         </is>
       </c>
       <c r="C23" s="11" t="n">
-        <v>1680.3</v>
+        <v>1699.03</v>
       </c>
       <c r="D23" s="15" t="n">
-        <v>202700190893</v>
+        <v>205204307648</v>
       </c>
       <c r="E23" s="15" t="n">
-        <v>6329745882</v>
-      </c>
-      <c r="F23" s="12" t="n">
-        <v>0.0061836</v>
+        <v>9085244988</v>
+      </c>
+      <c r="F23" s="16" t="n">
+        <v>0.0095683</v>
       </c>
       <c r="G23" s="10" t="inlineStr">
         <is>
-          <t>2026-06-13 21:39:57</t>
+          <t>2026-06-19 21:42:26</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="14" t="inlineStr">
         <is>
-          <t>Solana</t>
+          <t>Gram (prev. Toncoin)</t>
         </is>
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>SOL</t>
+          <t>GRAM</t>
         </is>
       </c>
       <c r="C24" s="11" t="n">
-        <v>68.22</v>
+        <v>1.65</v>
       </c>
       <c r="D24" s="15" t="n">
-        <v>39552259407</v>
+        <v>4436608700</v>
       </c>
       <c r="E24" s="15" t="n">
-        <v>1627493617</v>
+        <v>55639948</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>0.0139485</v>
+        <v>-0.0061558</v>
       </c>
       <c r="G24" s="10" t="inlineStr">
         <is>
-          <t>2026-06-13 21:39:57</t>
+          <t>2026-06-19 02:25:31</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="14" t="inlineStr">
         <is>
-          <t>Toncoin</t>
+          <t>Gram (prev. Toncoin)</t>
         </is>
       </c>
       <c r="B25" s="10" t="inlineStr">
         <is>
-          <t>TON</t>
+          <t>GRAM</t>
         </is>
       </c>
       <c r="C25" s="11" t="n">
-        <v>1.75</v>
+        <v>1.62</v>
       </c>
       <c r="D25" s="15" t="n">
-        <v>4678922525</v>
+        <v>4356775272</v>
       </c>
       <c r="E25" s="15" t="n">
-        <v>138169877</v>
+        <v>61320704</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>0.0251424</v>
+        <v>-0.0191556</v>
       </c>
       <c r="G25" s="10" t="inlineStr">
         <is>
-          <t>2026-06-13 21:39:57</t>
+          <t>2026-06-19 08:07:46</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="14" t="inlineStr">
         <is>
+          <t>Gram (prev. Toncoin)</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>GRAM</t>
+        </is>
+      </c>
+      <c r="C26" s="11" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="D26" s="15" t="n">
+        <v>4242911881</v>
+      </c>
+      <c r="E26" s="15" t="n">
+        <v>61666564</v>
+      </c>
+      <c r="F26" s="12" t="n">
+        <v>-0.039525</v>
+      </c>
+      <c r="G26" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-19 21:42:06</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="14" t="inlineStr">
+        <is>
+          <t>Gram (prev. Toncoin)</t>
+        </is>
+      </c>
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>GRAM</t>
+        </is>
+      </c>
+      <c r="C27" s="11" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="D27" s="15" t="n">
+        <v>4242911881</v>
+      </c>
+      <c r="E27" s="15" t="n">
+        <v>61666564</v>
+      </c>
+      <c r="F27" s="12" t="n">
+        <v>-0.039525</v>
+      </c>
+      <c r="G27" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-19 21:42:26</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="14" t="inlineStr">
+        <is>
           <t>NEAR Protocol</t>
         </is>
       </c>
-      <c r="B26" s="10" t="inlineStr">
+      <c r="B28" s="10" t="inlineStr">
         <is>
           <t>NEAR</t>
         </is>
       </c>
-      <c r="C26" s="11" t="n">
+      <c r="C28" s="11" t="n">
+        <v>2.03</v>
+      </c>
+      <c r="D28" s="15" t="n">
+        <v>2629686181</v>
+      </c>
+      <c r="E28" s="15" t="n">
+        <v>386759513</v>
+      </c>
+      <c r="F28" s="12" t="n">
+        <v>-0.0156479</v>
+      </c>
+      <c r="G28" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-12 22:36:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="14" t="inlineStr">
+        <is>
+          <t>NEAR Protocol</t>
+        </is>
+      </c>
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>NEAR</t>
+        </is>
+      </c>
+      <c r="C29" s="11" t="n">
+        <v>2.03</v>
+      </c>
+      <c r="D29" s="15" t="n">
+        <v>2629686181</v>
+      </c>
+      <c r="E29" s="15" t="n">
+        <v>386759513</v>
+      </c>
+      <c r="F29" s="12" t="n">
+        <v>-0.0156479</v>
+      </c>
+      <c r="G29" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-12 22:36:35</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="14" t="inlineStr">
+        <is>
+          <t>NEAR Protocol</t>
+        </is>
+      </c>
+      <c r="B30" s="10" t="inlineStr">
+        <is>
+          <t>NEAR</t>
+        </is>
+      </c>
+      <c r="C30" s="11" t="n">
+        <v>2.03</v>
+      </c>
+      <c r="D30" s="15" t="n">
+        <v>2638539801</v>
+      </c>
+      <c r="E30" s="15" t="n">
+        <v>387461086</v>
+      </c>
+      <c r="F30" s="12" t="n">
+        <v>-0.0137975</v>
+      </c>
+      <c r="G30" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-12 22:43:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="14" t="inlineStr">
+        <is>
+          <t>NEAR Protocol</t>
+        </is>
+      </c>
+      <c r="B31" s="10" t="inlineStr">
+        <is>
+          <t>NEAR</t>
+        </is>
+      </c>
+      <c r="C31" s="11" t="n">
+        <v>2.03</v>
+      </c>
+      <c r="D31" s="15" t="n">
+        <v>2638539801</v>
+      </c>
+      <c r="E31" s="15" t="n">
+        <v>387461086</v>
+      </c>
+      <c r="F31" s="12" t="n">
+        <v>-0.0137975</v>
+      </c>
+      <c r="G31" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-12 22:44:06</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="14" t="inlineStr">
+        <is>
+          <t>NEAR Protocol</t>
+        </is>
+      </c>
+      <c r="B32" s="10" t="inlineStr">
+        <is>
+          <t>NEAR</t>
+        </is>
+      </c>
+      <c r="C32" s="11" t="n">
         <v>2.12</v>
       </c>
-      <c r="D26" s="15" t="n">
+      <c r="D32" s="15" t="n">
         <v>2751683954</v>
       </c>
-      <c r="E26" s="15" t="n">
+      <c r="E32" s="15" t="n">
         <v>307118095</v>
       </c>
-      <c r="F26" s="12" t="n">
+      <c r="F32" s="16" t="n">
         <v>0.0424315</v>
       </c>
-      <c r="G26" s="10" t="inlineStr">
+      <c r="G32" s="10" t="inlineStr">
         <is>
           <t>2026-06-13 21:39:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="14" t="inlineStr">
+        <is>
+          <t>NEAR Protocol</t>
+        </is>
+      </c>
+      <c r="B33" s="10" t="inlineStr">
+        <is>
+          <t>NEAR</t>
+        </is>
+      </c>
+      <c r="C33" s="11" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="D33" s="15" t="n">
+        <v>2746473293</v>
+      </c>
+      <c r="E33" s="15" t="n">
+        <v>307334003</v>
+      </c>
+      <c r="F33" s="16" t="n">
+        <v>0.0453585</v>
+      </c>
+      <c r="G33" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-13 22:04:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="14" t="inlineStr">
+        <is>
+          <t>NEAR Protocol</t>
+        </is>
+      </c>
+      <c r="B34" s="10" t="inlineStr">
+        <is>
+          <t>NEAR</t>
+        </is>
+      </c>
+      <c r="C34" s="11" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="D34" s="15" t="n">
+        <v>3122784359</v>
+      </c>
+      <c r="E34" s="15" t="n">
+        <v>407916537</v>
+      </c>
+      <c r="F34" s="16" t="n">
+        <v>0.1344934</v>
+      </c>
+      <c r="G34" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-15 11:58:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="14" t="inlineStr">
+        <is>
+          <t>NEAR Protocol</t>
+        </is>
+      </c>
+      <c r="B35" s="10" t="inlineStr">
+        <is>
+          <t>NEAR</t>
+        </is>
+      </c>
+      <c r="C35" s="11" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="D35" s="15" t="n">
+        <v>2853008582</v>
+      </c>
+      <c r="E35" s="15" t="n">
+        <v>393241160</v>
+      </c>
+      <c r="F35" s="16" t="n">
+        <v>0.0025802</v>
+      </c>
+      <c r="G35" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-19 02:25:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="14" t="inlineStr">
+        <is>
+          <t>NEAR Protocol</t>
+        </is>
+      </c>
+      <c r="B36" s="10" t="inlineStr">
+        <is>
+          <t>NEAR</t>
+        </is>
+      </c>
+      <c r="C36" s="11" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="D36" s="15" t="n">
+        <v>2736312152</v>
+      </c>
+      <c r="E36" s="15" t="n">
+        <v>410116623</v>
+      </c>
+      <c r="F36" s="12" t="n">
+        <v>-0.0160383</v>
+      </c>
+      <c r="G36" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-19 08:07:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="14" t="inlineStr">
+        <is>
+          <t>NEAR Protocol</t>
+        </is>
+      </c>
+      <c r="B37" s="10" t="inlineStr">
+        <is>
+          <t>NEAR</t>
+        </is>
+      </c>
+      <c r="C37" s="11" t="n">
+        <v>2.14</v>
+      </c>
+      <c r="D37" s="15" t="n">
+        <v>2784698447</v>
+      </c>
+      <c r="E37" s="15" t="n">
+        <v>323980921</v>
+      </c>
+      <c r="F37" s="12" t="n">
+        <v>-0.0181993</v>
+      </c>
+      <c r="G37" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-19 21:42:06</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="14" t="inlineStr">
+        <is>
+          <t>NEAR Protocol</t>
+        </is>
+      </c>
+      <c r="B38" s="10" t="inlineStr">
+        <is>
+          <t>NEAR</t>
+        </is>
+      </c>
+      <c r="C38" s="11" t="n">
+        <v>2.14</v>
+      </c>
+      <c r="D38" s="15" t="n">
+        <v>2784698447</v>
+      </c>
+      <c r="E38" s="15" t="n">
+        <v>323980921</v>
+      </c>
+      <c r="F38" s="12" t="n">
+        <v>-0.0181993</v>
+      </c>
+      <c r="G38" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-19 21:42:26</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="14" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="B39" s="10" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C39" s="11" t="n">
+        <v>67.06999999999999</v>
+      </c>
+      <c r="D39" s="15" t="n">
+        <v>38891640092</v>
+      </c>
+      <c r="E39" s="15" t="n">
+        <v>2789772399</v>
+      </c>
+      <c r="F39" s="16" t="n">
+        <v>0.0002204</v>
+      </c>
+      <c r="G39" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-12 22:36:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="14" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="B40" s="10" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C40" s="11" t="n">
+        <v>67.06999999999999</v>
+      </c>
+      <c r="D40" s="15" t="n">
+        <v>38891640092</v>
+      </c>
+      <c r="E40" s="15" t="n">
+        <v>2789772399</v>
+      </c>
+      <c r="F40" s="16" t="n">
+        <v>0.0002204</v>
+      </c>
+      <c r="G40" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-12 22:36:35</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="14" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="B41" s="10" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C41" s="11" t="n">
+        <v>67.11</v>
+      </c>
+      <c r="D41" s="15" t="n">
+        <v>38918087648</v>
+      </c>
+      <c r="E41" s="15" t="n">
+        <v>2762112454</v>
+      </c>
+      <c r="F41" s="16" t="n">
+        <v>0.000721</v>
+      </c>
+      <c r="G41" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-12 22:43:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="14" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="B42" s="10" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C42" s="11" t="n">
+        <v>67.11</v>
+      </c>
+      <c r="D42" s="15" t="n">
+        <v>38918087648</v>
+      </c>
+      <c r="E42" s="15" t="n">
+        <v>2762112454</v>
+      </c>
+      <c r="F42" s="16" t="n">
+        <v>0.000721</v>
+      </c>
+      <c r="G42" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-12 22:44:06</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="14" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="B43" s="10" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C43" s="11" t="n">
+        <v>68.22</v>
+      </c>
+      <c r="D43" s="15" t="n">
+        <v>39552259407</v>
+      </c>
+      <c r="E43" s="15" t="n">
+        <v>1627493617</v>
+      </c>
+      <c r="F43" s="16" t="n">
+        <v>0.0139485</v>
+      </c>
+      <c r="G43" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-13 21:39:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="14" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="B44" s="10" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C44" s="11" t="n">
+        <v>68.09999999999999</v>
+      </c>
+      <c r="D44" s="15" t="n">
+        <v>39485251597</v>
+      </c>
+      <c r="E44" s="15" t="n">
+        <v>1612611692</v>
+      </c>
+      <c r="F44" s="16" t="n">
+        <v>0.0150488</v>
+      </c>
+      <c r="G44" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-13 22:04:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="14" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="B45" s="10" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C45" s="11" t="n">
+        <v>71.26000000000001</v>
+      </c>
+      <c r="D45" s="15" t="n">
+        <v>41343826608</v>
+      </c>
+      <c r="E45" s="15" t="n">
+        <v>1968842426</v>
+      </c>
+      <c r="F45" s="16" t="n">
+        <v>0.0449228</v>
+      </c>
+      <c r="G45" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-15 11:58:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="14" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="B46" s="10" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C46" s="11" t="n">
+        <v>69.39</v>
+      </c>
+      <c r="D46" s="15" t="n">
+        <v>40250816509</v>
+      </c>
+      <c r="E46" s="15" t="n">
+        <v>2416981074</v>
+      </c>
+      <c r="F46" s="12" t="n">
+        <v>-0.0364431</v>
+      </c>
+      <c r="G46" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-19 02:25:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="14" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="B47" s="10" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C47" s="11" t="n">
+        <v>68.48999999999999</v>
+      </c>
+      <c r="D47" s="15" t="n">
+        <v>39661175125</v>
+      </c>
+      <c r="E47" s="15" t="n">
+        <v>2493149286</v>
+      </c>
+      <c r="F47" s="12" t="n">
+        <v>-0.0335245</v>
+      </c>
+      <c r="G47" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-19 08:07:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="14" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="B48" s="10" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C48" s="11" t="n">
+        <v>68.81999999999999</v>
+      </c>
+      <c r="D48" s="15" t="n">
+        <v>40036132050</v>
+      </c>
+      <c r="E48" s="15" t="n">
+        <v>2025220338</v>
+      </c>
+      <c r="F48" s="16" t="n">
+        <v>0.0051467</v>
+      </c>
+      <c r="G48" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-19 21:42:06</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="14" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="B49" s="10" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C49" s="11" t="n">
+        <v>68.81999999999999</v>
+      </c>
+      <c r="D49" s="15" t="n">
+        <v>40036132050</v>
+      </c>
+      <c r="E49" s="15" t="n">
+        <v>2025220338</v>
+      </c>
+      <c r="F49" s="16" t="n">
+        <v>0.0051467</v>
+      </c>
+      <c r="G49" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-19 21:42:26</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="14" t="inlineStr">
+        <is>
+          <t>Toncoin</t>
+        </is>
+      </c>
+      <c r="B50" s="10" t="inlineStr">
+        <is>
+          <t>TON</t>
+        </is>
+      </c>
+      <c r="C50" s="11" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="D50" s="15" t="n">
+        <v>4496794507</v>
+      </c>
+      <c r="E50" s="15" t="n">
+        <v>228774793</v>
+      </c>
+      <c r="F50" s="12" t="n">
+        <v>-0.009129399999999999</v>
+      </c>
+      <c r="G50" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-12 22:36:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="14" t="inlineStr">
+        <is>
+          <t>Toncoin</t>
+        </is>
+      </c>
+      <c r="B51" s="10" t="inlineStr">
+        <is>
+          <t>TON</t>
+        </is>
+      </c>
+      <c r="C51" s="11" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="D51" s="15" t="n">
+        <v>4496794507</v>
+      </c>
+      <c r="E51" s="15" t="n">
+        <v>228774793</v>
+      </c>
+      <c r="F51" s="12" t="n">
+        <v>-0.009129399999999999</v>
+      </c>
+      <c r="G51" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-12 22:36:35</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="14" t="inlineStr">
+        <is>
+          <t>Toncoin</t>
+        </is>
+      </c>
+      <c r="B52" s="10" t="inlineStr">
+        <is>
+          <t>TON</t>
+        </is>
+      </c>
+      <c r="C52" s="11" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="D52" s="15" t="n">
+        <v>4505181149</v>
+      </c>
+      <c r="E52" s="15" t="n">
+        <v>229295333</v>
+      </c>
+      <c r="F52" s="12" t="n">
+        <v>-0.0063561</v>
+      </c>
+      <c r="G52" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-12 22:43:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="14" t="inlineStr">
+        <is>
+          <t>Toncoin</t>
+        </is>
+      </c>
+      <c r="B53" s="10" t="inlineStr">
+        <is>
+          <t>TON</t>
+        </is>
+      </c>
+      <c r="C53" s="11" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="D53" s="15" t="n">
+        <v>4505181149</v>
+      </c>
+      <c r="E53" s="15" t="n">
+        <v>229295333</v>
+      </c>
+      <c r="F53" s="12" t="n">
+        <v>-0.0063561</v>
+      </c>
+      <c r="G53" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-12 22:44:06</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="14" t="inlineStr">
+        <is>
+          <t>Toncoin</t>
+        </is>
+      </c>
+      <c r="B54" s="10" t="inlineStr">
+        <is>
+          <t>TON</t>
+        </is>
+      </c>
+      <c r="C54" s="11" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="D54" s="15" t="n">
+        <v>4678922525</v>
+      </c>
+      <c r="E54" s="15" t="n">
+        <v>138169877</v>
+      </c>
+      <c r="F54" s="16" t="n">
+        <v>0.0251424</v>
+      </c>
+      <c r="G54" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-13 21:39:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="14" t="inlineStr">
+        <is>
+          <t>Toncoin</t>
+        </is>
+      </c>
+      <c r="B55" s="10" t="inlineStr">
+        <is>
+          <t>TON</t>
+        </is>
+      </c>
+      <c r="C55" s="11" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="D55" s="15" t="n">
+        <v>4671728940</v>
+      </c>
+      <c r="E55" s="15" t="n">
+        <v>148188529</v>
+      </c>
+      <c r="F55" s="16" t="n">
+        <v>0.03329</v>
+      </c>
+      <c r="G55" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-13 22:04:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="14" t="inlineStr">
+        <is>
+          <t>Toncoin</t>
+        </is>
+      </c>
+      <c r="B56" s="10" t="inlineStr">
+        <is>
+          <t>TON</t>
+        </is>
+      </c>
+      <c r="C56" s="11" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="D56" s="15" t="n">
+        <v>4816929214</v>
+      </c>
+      <c r="E56" s="15" t="n">
+        <v>172079618</v>
+      </c>
+      <c r="F56" s="16" t="n">
+        <v>0.0465588</v>
+      </c>
+      <c r="G56" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-15 11:58:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="14" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="B57" s="10" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C57" s="11" t="n">
+        <v>63469</v>
+      </c>
+      <c r="D57" s="15" t="n">
+        <v>1271447224318</v>
+      </c>
+      <c r="E57" s="15" t="n">
+        <v>22319422351</v>
+      </c>
+      <c r="F57" s="16" t="n">
+        <v>0.012582</v>
+      </c>
+      <c r="G57" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-20 07:28:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="14" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="B58" s="10" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C58" s="11" t="n">
+        <v>1709.68</v>
+      </c>
+      <c r="D58" s="15" t="n">
+        <v>206125430978</v>
+      </c>
+      <c r="E58" s="15" t="n">
+        <v>6795533065</v>
+      </c>
+      <c r="F58" s="16" t="n">
+        <v>0.009428800000000001</v>
+      </c>
+      <c r="G58" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-20 07:28:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="14" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="B59" s="10" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C59" s="11" t="n">
+        <v>70.19</v>
+      </c>
+      <c r="D59" s="15" t="n">
+        <v>40697171192</v>
+      </c>
+      <c r="E59" s="15" t="n">
+        <v>1836186827</v>
+      </c>
+      <c r="F59" s="16" t="n">
+        <v>0.020042</v>
+      </c>
+      <c r="G59" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-20 07:28:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="14" t="inlineStr">
+        <is>
+          <t>Gram (prev. Toncoin)</t>
+        </is>
+      </c>
+      <c r="B60" s="10" t="inlineStr">
+        <is>
+          <t>GRAM</t>
+        </is>
+      </c>
+      <c r="C60" s="11" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="D60" s="15" t="n">
+        <v>4285385936</v>
+      </c>
+      <c r="E60" s="15" t="n">
+        <v>55073020</v>
+      </c>
+      <c r="F60" s="12" t="n">
+        <v>-0.0211067</v>
+      </c>
+      <c r="G60" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-20 07:28:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="14" t="inlineStr">
+        <is>
+          <t>NEAR Protocol</t>
+        </is>
+      </c>
+      <c r="B61" s="10" t="inlineStr">
+        <is>
+          <t>NEAR</t>
+        </is>
+      </c>
+      <c r="C61" s="11" t="n">
+        <v>2.17</v>
+      </c>
+      <c r="D61" s="15" t="n">
+        <v>2813799501</v>
+      </c>
+      <c r="E61" s="15" t="n">
+        <v>277490274</v>
+      </c>
+      <c r="F61" s="16" t="n">
+        <v>0.0168956</v>
+      </c>
+      <c r="G61" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-20 07:28:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="14" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="B62" s="10" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C62" s="11" t="n">
+        <v>64376</v>
+      </c>
+      <c r="D62" s="15" t="n">
+        <v>1290543361691</v>
+      </c>
+      <c r="E62" s="15" t="n">
+        <v>18446653854</v>
+      </c>
+      <c r="F62" s="16" t="n">
+        <v>0.0136434</v>
+      </c>
+      <c r="G62" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-21 07:51:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="14" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="B63" s="10" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C63" s="11" t="n">
+        <v>1734.72</v>
+      </c>
+      <c r="D63" s="15" t="n">
+        <v>209362468459</v>
+      </c>
+      <c r="E63" s="15" t="n">
+        <v>8366591493</v>
+      </c>
+      <c r="F63" s="16" t="n">
+        <v>0.013121</v>
+      </c>
+      <c r="G63" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-21 07:51:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="14" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="B64" s="10" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C64" s="11" t="n">
+        <v>73.59999999999999</v>
+      </c>
+      <c r="D64" s="15" t="n">
+        <v>42714106110</v>
+      </c>
+      <c r="E64" s="15" t="n">
+        <v>2220155349</v>
+      </c>
+      <c r="F64" s="16" t="n">
+        <v>0.038535</v>
+      </c>
+      <c r="G64" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-21 07:51:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="14" t="inlineStr">
+        <is>
+          <t>Gram (prev. Toncoin)</t>
+        </is>
+      </c>
+      <c r="B65" s="10" t="inlineStr">
+        <is>
+          <t>GRAM</t>
+        </is>
+      </c>
+      <c r="C65" s="11" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="D65" s="15" t="n">
+        <v>4428421216</v>
+      </c>
+      <c r="E65" s="15" t="n">
+        <v>32844164</v>
+      </c>
+      <c r="F65" s="16" t="n">
+        <v>0.03034</v>
+      </c>
+      <c r="G65" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-21 07:51:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="14" t="inlineStr">
+        <is>
+          <t>NEAR Protocol</t>
+        </is>
+      </c>
+      <c r="B66" s="10" t="inlineStr">
+        <is>
+          <t>NEAR</t>
+        </is>
+      </c>
+      <c r="C66" s="11" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="D66" s="15" t="n">
+        <v>2870804416</v>
+      </c>
+      <c r="E66" s="15" t="n">
+        <v>239256296</v>
+      </c>
+      <c r="F66" s="16" t="n">
+        <v>0.0182492</v>
+      </c>
+      <c r="G66" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-21 07:51:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="14" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="B67" s="10" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C67" s="11" t="n">
+        <v>63771</v>
+      </c>
+      <c r="D67" s="15" t="n">
+        <v>1278422396351</v>
+      </c>
+      <c r="E67" s="15" t="n">
+        <v>24322107125</v>
+      </c>
+      <c r="F67" s="12" t="n">
+        <v>-0.0022059</v>
+      </c>
+      <c r="G67" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-23 07:44:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="14" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="B68" s="10" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C68" s="11" t="n">
+        <v>1721.58</v>
+      </c>
+      <c r="D68" s="15" t="n">
+        <v>207763478376</v>
+      </c>
+      <c r="E68" s="15" t="n">
+        <v>12157462526</v>
+      </c>
+      <c r="F68" s="12" t="n">
+        <v>-0.005202599999999999</v>
+      </c>
+      <c r="G68" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-23 07:44:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="14" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="B69" s="10" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C69" s="11" t="n">
+        <v>71.70999999999999</v>
+      </c>
+      <c r="D69" s="15" t="n">
+        <v>41648637560</v>
+      </c>
+      <c r="E69" s="15" t="n">
+        <v>2347306271</v>
+      </c>
+      <c r="F69" s="12" t="n">
+        <v>-0.0232903</v>
+      </c>
+      <c r="G69" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-23 07:44:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="14" t="inlineStr">
+        <is>
+          <t>Gram (prev. Toncoin)</t>
+        </is>
+      </c>
+      <c r="B70" s="10" t="inlineStr">
+        <is>
+          <t>GRAM</t>
+        </is>
+      </c>
+      <c r="C70" s="11" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="D70" s="15" t="n">
+        <v>4541430837</v>
+      </c>
+      <c r="E70" s="15" t="n">
+        <v>5807509</v>
+      </c>
+      <c r="F70" s="16" t="n">
+        <v>0.0354824</v>
+      </c>
+      <c r="G70" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-23 07:44:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="14" t="inlineStr">
+        <is>
+          <t>NEAR Protocol</t>
+        </is>
+      </c>
+      <c r="B71" s="10" t="inlineStr">
+        <is>
+          <t>NEAR</t>
+        </is>
+      </c>
+      <c r="C71" s="11" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="D71" s="15" t="n">
+        <v>2669312890</v>
+      </c>
+      <c r="E71" s="15" t="n">
+        <v>294238843</v>
+      </c>
+      <c r="F71" s="12" t="n">
+        <v>-0.04123300000000001</v>
+      </c>
+      <c r="G71" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-23 07:44:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="14" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="B72" s="10" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C72" s="11" t="n">
+        <v>62698</v>
+      </c>
+      <c r="D72" s="15" t="n">
+        <v>1256691097933</v>
+      </c>
+      <c r="E72" s="15" t="n">
+        <v>30181000165</v>
+      </c>
+      <c r="F72" s="12" t="n">
+        <v>-0.0147875</v>
+      </c>
+      <c r="G72" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-24 07:51:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="14" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="B73" s="10" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C73" s="11" t="n">
+        <v>1667.47</v>
+      </c>
+      <c r="D73" s="15" t="n">
+        <v>201153373337</v>
+      </c>
+      <c r="E73" s="15" t="n">
+        <v>10545751042</v>
+      </c>
+      <c r="F73" s="12" t="n">
+        <v>-0.0298031</v>
+      </c>
+      <c r="G73" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-24 07:51:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="14" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="B74" s="10" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C74" s="11" t="n">
+        <v>69.47</v>
+      </c>
+      <c r="D74" s="15" t="n">
+        <v>40295883261</v>
+      </c>
+      <c r="E74" s="15" t="n">
+        <v>2284359145</v>
+      </c>
+      <c r="F74" s="12" t="n">
+        <v>-0.027861</v>
+      </c>
+      <c r="G74" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-24 07:51:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="14" t="inlineStr">
+        <is>
+          <t>Gram (prev. Toncoin)</t>
+        </is>
+      </c>
+      <c r="B75" s="10" t="inlineStr">
+        <is>
+          <t>GRAM</t>
+        </is>
+      </c>
+      <c r="C75" s="11" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="D75" s="15" t="n">
+        <v>4197039565</v>
+      </c>
+      <c r="E75" s="15" t="n">
+        <v>12268958</v>
+      </c>
+      <c r="F75" s="12" t="n">
+        <v>-0.08046110000000001</v>
+      </c>
+      <c r="G75" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-24 07:51:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="14" t="inlineStr">
+        <is>
+          <t>NEAR Protocol</t>
+        </is>
+      </c>
+      <c r="B76" s="10" t="inlineStr">
+        <is>
+          <t>NEAR</t>
+        </is>
+      </c>
+      <c r="C76" s="11" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="D76" s="15" t="n">
+        <v>2550289042</v>
+      </c>
+      <c r="E76" s="15" t="n">
+        <v>234710051</v>
+      </c>
+      <c r="F76" s="12" t="n">
+        <v>-0.0311822</v>
+      </c>
+      <c r="G76" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-24 07:51:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="14" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="B77" s="10" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C77" s="11" t="n">
+        <v>60750</v>
+      </c>
+      <c r="D77" s="15" t="n">
+        <v>1217903576423</v>
+      </c>
+      <c r="E77" s="15" t="n">
+        <v>41220920517</v>
+      </c>
+      <c r="F77" s="12" t="n">
+        <v>-0.0293159</v>
+      </c>
+      <c r="G77" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-25 07:14:43</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="14" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="B78" s="10" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C78" s="11" t="n">
+        <v>1616.54</v>
+      </c>
+      <c r="D78" s="15" t="n">
+        <v>195078928735</v>
+      </c>
+      <c r="E78" s="15" t="n">
+        <v>14103500766</v>
+      </c>
+      <c r="F78" s="12" t="n">
+        <v>-0.0279496</v>
+      </c>
+      <c r="G78" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-25 07:14:43</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="14" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="B79" s="10" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C79" s="11" t="n">
+        <v>67.54000000000001</v>
+      </c>
+      <c r="D79" s="15" t="n">
+        <v>39210479653</v>
+      </c>
+      <c r="E79" s="15" t="n">
+        <v>3196392733</v>
+      </c>
+      <c r="F79" s="12" t="n">
+        <v>-0.026841</v>
+      </c>
+      <c r="G79" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-25 07:14:43</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="14" t="inlineStr">
+        <is>
+          <t>Gram (prev. Toncoin)</t>
+        </is>
+      </c>
+      <c r="B80" s="10" t="inlineStr">
+        <is>
+          <t>GRAM</t>
+        </is>
+      </c>
+      <c r="C80" s="11" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="D80" s="15" t="n">
+        <v>4287944981</v>
+      </c>
+      <c r="E80" s="15" t="n">
+        <v>5122663</v>
+      </c>
+      <c r="F80" s="16" t="n">
+        <v>0.0254335</v>
+      </c>
+      <c r="G80" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-25 07:14:43</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="14" t="inlineStr">
+        <is>
+          <t>NEAR Protocol</t>
+        </is>
+      </c>
+      <c r="B81" s="10" t="inlineStr">
+        <is>
+          <t>NEAR</t>
+        </is>
+      </c>
+      <c r="C81" s="11" t="n">
+        <v>1.94</v>
+      </c>
+      <c r="D81" s="15" t="n">
+        <v>2517498630</v>
+      </c>
+      <c r="E81" s="15" t="n">
+        <v>254607787</v>
+      </c>
+      <c r="F81" s="12" t="n">
+        <v>-0.0120728</v>
+      </c>
+      <c r="G81" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-25 07:14:43</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="14" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="B82" s="10" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C82" s="11" t="n">
+        <v>59817</v>
+      </c>
+      <c r="D82" s="15" t="n">
+        <v>1199185701665</v>
+      </c>
+      <c r="E82" s="15" t="n">
+        <v>44950307488</v>
+      </c>
+      <c r="F82" s="12" t="n">
+        <v>-0.0270187</v>
+      </c>
+      <c r="G82" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-26 08:45:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="14" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="B83" s="10" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C83" s="11" t="n">
+        <v>1553.31</v>
+      </c>
+      <c r="D83" s="15" t="n">
+        <v>187470573659</v>
+      </c>
+      <c r="E83" s="15" t="n">
+        <v>16575808924</v>
+      </c>
+      <c r="F83" s="12" t="n">
+        <v>-0.0549016</v>
+      </c>
+      <c r="G83" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-26 08:45:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="14" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="B84" s="10" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C84" s="11" t="n">
+        <v>68.20999999999999</v>
+      </c>
+      <c r="D84" s="15" t="n">
+        <v>39614309180</v>
+      </c>
+      <c r="E84" s="15" t="n">
+        <v>3821229254</v>
+      </c>
+      <c r="F84" s="12" t="n">
+        <v>-0.0121682</v>
+      </c>
+      <c r="G84" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-26 08:45:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="14" t="inlineStr">
+        <is>
+          <t>Gram (prev. Toncoin)</t>
+        </is>
+      </c>
+      <c r="B85" s="10" t="inlineStr">
+        <is>
+          <t>GRAM</t>
+        </is>
+      </c>
+      <c r="C85" s="11" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="D85" s="15" t="n">
+        <v>4249207381</v>
+      </c>
+      <c r="E85" s="15" t="n">
+        <v>4560983</v>
+      </c>
+      <c r="F85" s="12" t="n">
+        <v>-0.0091939</v>
+      </c>
+      <c r="G85" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-26 08:45:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="14" t="inlineStr">
+        <is>
+          <t>NEAR Protocol</t>
+        </is>
+      </c>
+      <c r="B86" s="10" t="inlineStr">
+        <is>
+          <t>NEAR</t>
+        </is>
+      </c>
+      <c r="C86" s="11" t="n">
+        <v>1.81</v>
+      </c>
+      <c r="D86" s="15" t="n">
+        <v>2350850750</v>
+      </c>
+      <c r="E86" s="15" t="n">
+        <v>355820934</v>
+      </c>
+      <c r="F86" s="12" t="n">
+        <v>-0.07882209999999999</v>
+      </c>
+      <c r="G86" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-26 08:45:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="14" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="B87" s="10" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C87" s="11" t="n">
+        <v>59376</v>
+      </c>
+      <c r="D87" s="15" t="n">
+        <v>1190565920546</v>
+      </c>
+      <c r="E87" s="15" t="n">
+        <v>30120258404</v>
+      </c>
+      <c r="F87" s="12" t="n">
+        <v>-0.0075148</v>
+      </c>
+      <c r="G87" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-30 07:10:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="14" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="B88" s="10" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C88" s="11" t="n">
+        <v>1579.66</v>
+      </c>
+      <c r="D88" s="15" t="n">
+        <v>190669965469</v>
+      </c>
+      <c r="E88" s="15" t="n">
+        <v>10725789113</v>
+      </c>
+      <c r="F88" s="16" t="n">
+        <v>0.0012383</v>
+      </c>
+      <c r="G88" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-30 07:10:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="14" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="B89" s="10" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C89" s="11" t="n">
+        <v>73.97</v>
+      </c>
+      <c r="D89" s="15" t="n">
+        <v>42965727340</v>
+      </c>
+      <c r="E89" s="15" t="n">
+        <v>3867086811</v>
+      </c>
+      <c r="F89" s="16" t="n">
+        <v>0.0200858</v>
+      </c>
+      <c r="G89" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-30 07:10:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="14" t="inlineStr">
+        <is>
+          <t>Gram (prev. Toncoin)</t>
+        </is>
+      </c>
+      <c r="B90" s="10" t="inlineStr">
+        <is>
+          <t>GRAM</t>
+        </is>
+      </c>
+      <c r="C90" s="11" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="D90" s="15" t="n">
+        <v>4317860633</v>
+      </c>
+      <c r="E90" s="15" t="n">
+        <v>2667265</v>
+      </c>
+      <c r="F90" s="16" t="n">
+        <v>0.000576</v>
+      </c>
+      <c r="G90" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-30 07:10:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="14" t="inlineStr">
+        <is>
+          <t>NEAR Protocol</t>
+        </is>
+      </c>
+      <c r="B91" s="10" t="inlineStr">
+        <is>
+          <t>NEAR</t>
+        </is>
+      </c>
+      <c r="C91" s="11" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="D91" s="15" t="n">
+        <v>2400460759</v>
+      </c>
+      <c r="E91" s="15" t="n">
+        <v>220965921</v>
+      </c>
+      <c r="F91" s="12" t="n">
+        <v>-0.007585199999999999</v>
+      </c>
+      <c r="G91" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-30 07:10:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="14" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="B92" s="10" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C92" s="11" t="n">
+        <v>60705</v>
+      </c>
+      <c r="D92" s="15" t="n">
+        <v>1217195726232</v>
+      </c>
+      <c r="E92" s="15" t="n">
+        <v>38818474558</v>
+      </c>
+      <c r="F92" s="16" t="n">
+        <v>0.0247862</v>
+      </c>
+      <c r="G92" s="10" t="inlineStr">
+        <is>
+          <t>2026-07-02 07:51:32</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="14" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="B93" s="10" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C93" s="11" t="n">
+        <v>1630.03</v>
+      </c>
+      <c r="D93" s="15" t="n">
+        <v>196716819686</v>
+      </c>
+      <c r="E93" s="15" t="n">
+        <v>11138200342</v>
+      </c>
+      <c r="F93" s="16" t="n">
+        <v>0.0207649</v>
+      </c>
+      <c r="G93" s="10" t="inlineStr">
+        <is>
+          <t>2026-07-02 07:51:32</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="14" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="B94" s="10" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C94" s="11" t="n">
+        <v>78.15000000000001</v>
+      </c>
+      <c r="D94" s="15" t="n">
+        <v>45379870220</v>
+      </c>
+      <c r="E94" s="15" t="n">
+        <v>3494448837</v>
+      </c>
+      <c r="F94" s="16" t="n">
+        <v>0.0339992</v>
+      </c>
+      <c r="G94" s="10" t="inlineStr">
+        <is>
+          <t>2026-07-02 07:51:32</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="14" t="inlineStr">
+        <is>
+          <t>Gram (prev. Toncoin)</t>
+        </is>
+      </c>
+      <c r="B95" s="10" t="inlineStr">
+        <is>
+          <t>GRAM</t>
+        </is>
+      </c>
+      <c r="C95" s="11" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="D95" s="15" t="n">
+        <v>4227715963</v>
+      </c>
+      <c r="E95" s="15" t="n">
+        <v>27102950</v>
+      </c>
+      <c r="F95" s="16" t="n">
+        <v>0.001453</v>
+      </c>
+      <c r="G95" s="10" t="inlineStr">
+        <is>
+          <t>2026-07-02 07:51:32</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="14" t="inlineStr">
+        <is>
+          <t>NEAR Protocol</t>
+        </is>
+      </c>
+      <c r="B96" s="10" t="inlineStr">
+        <is>
+          <t>NEAR</t>
+        </is>
+      </c>
+      <c r="C96" s="11" t="n">
+        <v>1.92</v>
+      </c>
+      <c r="D96" s="15" t="n">
+        <v>2489623194</v>
+      </c>
+      <c r="E96" s="15" t="n">
+        <v>283034150</v>
+      </c>
+      <c r="F96" s="16" t="n">
+        <v>0.0380796</v>
+      </c>
+      <c r="G96" s="10" t="inlineStr">
+        <is>
+          <t>2026-07-02 07:51:32</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="14" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="B97" s="10" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C97" s="11" t="n">
+        <v>63306</v>
+      </c>
+      <c r="D97" s="15" t="n">
+        <v>1269737068319</v>
+      </c>
+      <c r="E97" s="15" t="n">
+        <v>37908556696</v>
+      </c>
+      <c r="F97" s="16" t="n">
+        <v>0.0065796</v>
+      </c>
+      <c r="G97" s="10" t="inlineStr">
+        <is>
+          <t>2026-07-07 10:07:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="14" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="B98" s="10" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C98" s="11" t="n">
+        <v>1777.92</v>
+      </c>
+      <c r="D98" s="15" t="n">
+        <v>214598447518</v>
+      </c>
+      <c r="E98" s="15" t="n">
+        <v>16056538921</v>
+      </c>
+      <c r="F98" s="16" t="n">
+        <v>0.0050656</v>
+      </c>
+      <c r="G98" s="10" t="inlineStr">
+        <is>
+          <t>2026-07-07 10:07:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="14" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="B99" s="10" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C99" s="11" t="n">
+        <v>81.52</v>
+      </c>
+      <c r="D99" s="15" t="n">
+        <v>47437831868</v>
+      </c>
+      <c r="E99" s="15" t="n">
+        <v>2588321889</v>
+      </c>
+      <c r="F99" s="16" t="n">
+        <v>0.0155147</v>
+      </c>
+      <c r="G99" s="10" t="inlineStr">
+        <is>
+          <t>2026-07-07 10:07:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="14" t="inlineStr">
+        <is>
+          <t>Gram (prev. Toncoin)</t>
+        </is>
+      </c>
+      <c r="B100" s="10" t="inlineStr">
+        <is>
+          <t>GRAM</t>
+        </is>
+      </c>
+      <c r="C100" s="11" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="D100" s="15" t="n">
+        <v>4584759141</v>
+      </c>
+      <c r="E100" s="15" t="n">
+        <v>106715786</v>
+      </c>
+      <c r="F100" s="12" t="n">
+        <v>-0.0387627</v>
+      </c>
+      <c r="G100" s="10" t="inlineStr">
+        <is>
+          <t>2026-07-07 10:07:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="14" t="inlineStr">
+        <is>
+          <t>NEAR Protocol</t>
+        </is>
+      </c>
+      <c r="B101" s="10" t="inlineStr">
+        <is>
+          <t>NEAR</t>
+        </is>
+      </c>
+      <c r="C101" s="11" t="n">
+        <v>2.02</v>
+      </c>
+      <c r="D101" s="15" t="n">
+        <v>2628034551</v>
+      </c>
+      <c r="E101" s="15" t="n">
+        <v>284509160</v>
+      </c>
+      <c r="F101" s="16" t="n">
+        <v>0.0200752</v>
+      </c>
+      <c r="G101" s="10" t="inlineStr">
+        <is>
+          <t>2026-07-07 10:07:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="14" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="B102" s="10" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C102" s="11" t="n">
+        <v>62624</v>
+      </c>
+      <c r="D102" s="15" t="n">
+        <v>1255830689447</v>
+      </c>
+      <c r="E102" s="15" t="n">
+        <v>30892741610</v>
+      </c>
+      <c r="F102" s="12" t="n">
+        <v>-0.0108589</v>
+      </c>
+      <c r="G102" s="10" t="inlineStr">
+        <is>
+          <t>2026-07-08 09:51:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="14" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="B103" s="10" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C103" s="11" t="n">
+        <v>1750.74</v>
+      </c>
+      <c r="D103" s="15" t="n">
+        <v>211284626828</v>
+      </c>
+      <c r="E103" s="15" t="n">
+        <v>9954660898</v>
+      </c>
+      <c r="F103" s="12" t="n">
+        <v>-0.0160442</v>
+      </c>
+      <c r="G103" s="10" t="inlineStr">
+        <is>
+          <t>2026-07-08 09:51:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="14" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="B104" s="10" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C104" s="11" t="n">
+        <v>78.09</v>
+      </c>
+      <c r="D104" s="15" t="n">
+        <v>45424263956</v>
+      </c>
+      <c r="E104" s="15" t="n">
+        <v>2374583178</v>
+      </c>
+      <c r="F104" s="12" t="n">
+        <v>-0.04008130000000001</v>
+      </c>
+      <c r="G104" s="10" t="inlineStr">
+        <is>
+          <t>2026-07-08 09:51:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="14" t="inlineStr">
+        <is>
+          <t>Gram (prev. Toncoin)</t>
+        </is>
+      </c>
+      <c r="B105" s="10" t="inlineStr">
+        <is>
+          <t>GRAM</t>
+        </is>
+      </c>
+      <c r="C105" s="11" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="D105" s="15" t="n">
+        <v>4333611851</v>
+      </c>
+      <c r="E105" s="15" t="n">
+        <v>166937000</v>
+      </c>
+      <c r="F105" s="12" t="n">
+        <v>-0.0559572</v>
+      </c>
+      <c r="G105" s="10" t="inlineStr">
+        <is>
+          <t>2026-07-08 09:51:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="14" t="inlineStr">
+        <is>
+          <t>NEAR Protocol</t>
+        </is>
+      </c>
+      <c r="B106" s="10" t="inlineStr">
+        <is>
+          <t>NEAR</t>
+        </is>
+      </c>
+      <c r="C106" s="11" t="n">
+        <v>1.91</v>
+      </c>
+      <c r="D106" s="15" t="n">
+        <v>2479912954</v>
+      </c>
+      <c r="E106" s="15" t="n">
+        <v>249813935</v>
+      </c>
+      <c r="F106" s="12" t="n">
+        <v>-0.0544447</v>
+      </c>
+      <c r="G106" s="10" t="inlineStr">
+        <is>
+          <t>2026-07-08 09:51:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="14" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="B107" s="10" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C107" s="11" t="n">
+        <v>63965</v>
+      </c>
+      <c r="D107" s="15" t="n">
+        <v>1283072963270</v>
+      </c>
+      <c r="E107" s="15" t="n">
+        <v>17669729990</v>
+      </c>
+      <c r="F107" s="12" t="n">
+        <v>-0.001749</v>
+      </c>
+      <c r="G107" s="10" t="inlineStr">
+        <is>
+          <t>2026-07-12 07:50:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="14" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="B108" s="10" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C108" s="11" t="n">
+        <v>1805.25</v>
+      </c>
+      <c r="D108" s="15" t="n">
+        <v>217872077617</v>
+      </c>
+      <c r="E108" s="15" t="n">
+        <v>7347215508</v>
+      </c>
+      <c r="F108" s="16" t="n">
+        <v>0.0058596</v>
+      </c>
+      <c r="G108" s="10" t="inlineStr">
+        <is>
+          <t>2026-07-12 07:50:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="14" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="B109" s="10" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C109" s="11" t="n">
+        <v>76.7</v>
+      </c>
+      <c r="D109" s="15" t="n">
+        <v>44652305998</v>
+      </c>
+      <c r="E109" s="15" t="n">
+        <v>1451702561</v>
+      </c>
+      <c r="F109" s="12" t="n">
+        <v>-0.0133883</v>
+      </c>
+      <c r="G109" s="10" t="inlineStr">
+        <is>
+          <t>2026-07-12 07:50:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="14" t="inlineStr">
+        <is>
+          <t>Gram (prev. Toncoin)</t>
+        </is>
+      </c>
+      <c r="B110" s="10" t="inlineStr">
+        <is>
+          <t>GRAM</t>
+        </is>
+      </c>
+      <c r="C110" s="11" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="D110" s="15" t="n">
+        <v>4496165373</v>
+      </c>
+      <c r="E110" s="15" t="n">
+        <v>27919020</v>
+      </c>
+      <c r="F110" s="16" t="n">
+        <v>0.0096688</v>
+      </c>
+      <c r="G110" s="10" t="inlineStr">
+        <is>
+          <t>2026-07-12 07:50:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="14" t="inlineStr">
+        <is>
+          <t>NEAR Protocol</t>
+        </is>
+      </c>
+      <c r="B111" s="10" t="inlineStr">
+        <is>
+          <t>NEAR</t>
+        </is>
+      </c>
+      <c r="C111" s="11" t="n">
+        <v>1.89</v>
+      </c>
+      <c r="D111" s="15" t="n">
+        <v>2460377871</v>
+      </c>
+      <c r="E111" s="15" t="n">
+        <v>97694976</v>
+      </c>
+      <c r="F111" s="12" t="n">
+        <v>-0.0056801</v>
+      </c>
+      <c r="G111" s="10" t="inlineStr">
+        <is>
+          <t>2026-07-12 07:50:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="14" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="B112" s="10" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C112" s="11" t="n">
+        <v>62707</v>
+      </c>
+      <c r="D112" s="15" t="n">
+        <v>1257629626755</v>
+      </c>
+      <c r="E112" s="15" t="n">
+        <v>20788529125</v>
+      </c>
+      <c r="F112" s="12" t="n">
+        <v>-0.0196678</v>
+      </c>
+      <c r="G112" s="10" t="inlineStr">
+        <is>
+          <t>2026-07-13 08:08:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="14" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="B113" s="10" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C113" s="11" t="n">
+        <v>1782.08</v>
+      </c>
+      <c r="D113" s="15" t="n">
+        <v>215066098027</v>
+      </c>
+      <c r="E113" s="15" t="n">
+        <v>7273023289</v>
+      </c>
+      <c r="F113" s="12" t="n">
+        <v>-0.0125042</v>
+      </c>
+      <c r="G113" s="10" t="inlineStr">
+        <is>
+          <t>2026-07-13 08:08:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="14" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="B114" s="10" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C114" s="11" t="n">
+        <v>76.09</v>
+      </c>
+      <c r="D114" s="15" t="n">
+        <v>44305388486</v>
+      </c>
+      <c r="E114" s="15" t="n">
+        <v>1373848686</v>
+      </c>
+      <c r="F114" s="12" t="n">
+        <v>-0.0079445</v>
+      </c>
+      <c r="G114" s="10" t="inlineStr">
+        <is>
+          <t>2026-07-13 08:08:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="14" t="inlineStr">
+        <is>
+          <t>Gram (prev. Toncoin)</t>
+        </is>
+      </c>
+      <c r="B115" s="10" t="inlineStr">
+        <is>
+          <t>GRAM</t>
+        </is>
+      </c>
+      <c r="C115" s="11" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="D115" s="15" t="n">
+        <v>4358363128</v>
+      </c>
+      <c r="E115" s="15" t="n">
+        <v>23864724</v>
+      </c>
+      <c r="F115" s="12" t="n">
+        <v>-0.0334631</v>
+      </c>
+      <c r="G115" s="10" t="inlineStr">
+        <is>
+          <t>2026-07-13 08:08:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="14" t="inlineStr">
+        <is>
+          <t>NEAR Protocol</t>
+        </is>
+      </c>
+      <c r="B116" s="10" t="inlineStr">
+        <is>
+          <t>NEAR</t>
+        </is>
+      </c>
+      <c r="C116" s="11" t="n">
+        <v>1.87</v>
+      </c>
+      <c r="D116" s="15" t="n">
+        <v>2431223218</v>
+      </c>
+      <c r="E116" s="15" t="n">
+        <v>116891270</v>
+      </c>
+      <c r="F116" s="12" t="n">
+        <v>-0.010475</v>
+      </c>
+      <c r="G116" s="10" t="inlineStr">
+        <is>
+          <t>2026-07-13 08:08:00</t>
         </is>
       </c>
     </row>

</xml_diff>